<commit_message>
Doc: Adicionei os custos, requisitos da insfraestrutura, regra de negócio, história do usuário ao escopo e atualizei o cronograma
</commit_message>
<xml_diff>
--- a/Arquivos-Escopo/CRONOGRAMA_E_GRAFICO_FAZENDA_xlsx.xlsx
+++ b/Arquivos-Escopo/CRONOGRAMA_E_GRAFICO_FAZENDA_xlsx.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\OneDrive - SESISENAISP - Escolas\Área de Trabalho\AgroFlux2026\Arquivos-Escopo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DEDCEE-3E17-4404-B1B4-3BCCC35E73C9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{23DEDCEE-3E17-4404-B1B4-3BCCC35E73C9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{4831AF56-479A-451C-A882-7AA7681BE124}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{D227F423-1045-4383-BB6A-309B4CAF3E1E}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" activeTab="1" xr2:uid="{D227F423-1045-4383-BB6A-309B4CAF3E1E}"/>
   </bookViews>
   <sheets>
     <sheet name="RELATÓRIO DO CRONOGRAMA" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
   <si>
     <t>CRONOGRAMA</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Cronograma</t>
   </si>
   <si>
-    <t>Lista de materiais e equipamentos</t>
-  </si>
-  <si>
     <t>SPRINT 02</t>
   </si>
   <si>
@@ -62,9 +59,6 @@
   </si>
   <si>
     <t>Documentação final</t>
-  </si>
-  <si>
-    <t>PROGRESSO</t>
   </si>
   <si>
     <t xml:space="preserve">Levantamento de requisitos </t>
@@ -105,15 +99,12 @@
   <si>
     <t xml:space="preserve">CONCLUIDO </t>
   </si>
-  <si>
-    <t xml:space="preserve">PROGRESSO </t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,13 +116,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -267,26 +251,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -313,18 +291,33 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+  <dxfs count="213">
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -334,6 +327,1957 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFB7B7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9393"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6D6D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FF8D8A0D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FFB3AF11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FFB3AF11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE3EB81"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FFBEBA12"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2EA7E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FFFFCC00"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2EA7E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color rgb="FFFFFF00"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7E24A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7E24A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7E24A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7E24A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
@@ -462,6 +2406,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -469,12 +2420,16 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FFFEFC9C"/>
-      <color rgb="FF74F87A"/>
-      <color rgb="FFFCD0E0"/>
-      <color rgb="FFFBBBD2"/>
-      <color rgb="FFFDE7EF"/>
-      <color rgb="FFF7C9E7"/>
+      <color rgb="FFFFB7B7"/>
+      <color rgb="FFFF9393"/>
+      <color rgb="FFFF6D6D"/>
+      <color rgb="FF8D8A0D"/>
+      <color rgb="FFE3EB81"/>
+      <color rgb="FFB3AF11"/>
+      <color rgb="FFBEBA12"/>
+      <color rgb="FFE2EA7E"/>
+      <color rgb="FFFFCC00"/>
+      <color rgb="FFD7E24A"/>
     </mruColors>
   </colors>
   <extLst>
@@ -544,16 +2499,16 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$C$22</c15:sqref>
+                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$C$21</c15:sqref>
                   </c15:fullRef>
                   <c15:levelRef>
-                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$22</c15:sqref>
+                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$21</c15:sqref>
                   </c15:levelRef>
                 </c:ext>
               </c:extLst>
-              <c:f>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$22</c:f>
+              <c:f>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$21</c:f>
               <c:strCache>
-                <c:ptCount val="18"/>
+                <c:ptCount val="17"/>
                 <c:pt idx="0">
                   <c:v>Levantamento de requisitos </c:v>
                 </c:pt>
@@ -564,48 +2519,45 @@
                   <c:v>Cronograma</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Lista de materiais e equipamentos</c:v>
+                  <c:v>Cronograma</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Cronograma</c:v>
+                  <c:v>Custos do projeto</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Custos do projeto</c:v>
+                  <c:v>Desenvolvimento da Introdução do Relatório Técnico</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Desenvolvimento da Introdução do Relatório Técnico</c:v>
+                  <c:v>SPRINT 02</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>SPRINT 02</c:v>
+                  <c:v>Wireframe de Alta Fidelidade</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Wireframe de Alta Fidelidade</c:v>
+                  <c:v>Front-End do Projeto</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Front-End do Projeto</c:v>
+                  <c:v>Desenvolvimento da Metodologia do Relatório Técnico.</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Desenvolvimento da Metodologia do Relatório Técnico.</c:v>
+                  <c:v>SPRINT 03</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>SPRINT 03</c:v>
+                  <c:v>Programação Back-End</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Programação Back-End</c:v>
+                  <c:v>Código fonte do programa</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Código fonte do programa</c:v>
+                  <c:v>Documentação final</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>Documentação final</c:v>
+                  <c:v>SPRINT 04</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>SPRINT 04</c:v>
+                  <c:v>Projeto Final do Semestre</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>Projeto Final do Semestre</c:v>
-                </c:pt>
-                <c:pt idx="17">
                   <c:v>Relatório Final.</c:v>
                 </c:pt>
               </c:strCache>
@@ -613,29 +2565,29 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'RELATÓRIO DO CRONOGRAMA'!$D$5:$D$22</c:f>
+              <c:f>'RELATÓRIO DO CRONOGRAMA'!$D$5:$D$21</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="17"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
@@ -644,7 +2596,7 @@
                 <c:pt idx="9">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
@@ -653,13 +2605,10 @@
                 <c:pt idx="13">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="15">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="17">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -706,16 +2655,16 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$C$22</c15:sqref>
+                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$C$21</c15:sqref>
                   </c15:fullRef>
                   <c15:levelRef>
-                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$22</c15:sqref>
+                    <c15:sqref>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$21</c15:sqref>
                   </c15:levelRef>
                 </c:ext>
               </c:extLst>
-              <c:f>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$22</c:f>
+              <c:f>'RELATÓRIO DO CRONOGRAMA'!$B$5:$B$21</c:f>
               <c:strCache>
-                <c:ptCount val="18"/>
+                <c:ptCount val="17"/>
                 <c:pt idx="0">
                   <c:v>Levantamento de requisitos </c:v>
                 </c:pt>
@@ -726,48 +2675,45 @@
                   <c:v>Cronograma</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Lista de materiais e equipamentos</c:v>
+                  <c:v>Cronograma</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Cronograma</c:v>
+                  <c:v>Custos do projeto</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Custos do projeto</c:v>
+                  <c:v>Desenvolvimento da Introdução do Relatório Técnico</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Desenvolvimento da Introdução do Relatório Técnico</c:v>
+                  <c:v>SPRINT 02</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>SPRINT 02</c:v>
+                  <c:v>Wireframe de Alta Fidelidade</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Wireframe de Alta Fidelidade</c:v>
+                  <c:v>Front-End do Projeto</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Front-End do Projeto</c:v>
+                  <c:v>Desenvolvimento da Metodologia do Relatório Técnico.</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Desenvolvimento da Metodologia do Relatório Técnico.</c:v>
+                  <c:v>SPRINT 03</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>SPRINT 03</c:v>
+                  <c:v>Programação Back-End</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Programação Back-End</c:v>
+                  <c:v>Código fonte do programa</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Código fonte do programa</c:v>
+                  <c:v>Documentação final</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>Documentação final</c:v>
+                  <c:v>SPRINT 04</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>SPRINT 04</c:v>
+                  <c:v>Projeto Final do Semestre</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>Projeto Final do Semestre</c:v>
-                </c:pt>
-                <c:pt idx="17">
                   <c:v>Relatório Final.</c:v>
                 </c:pt>
               </c:strCache>
@@ -775,10 +2721,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'RELATÓRIO DO CRONOGRAMA'!$E$5:$E$22</c:f>
+              <c:f>'RELATÓRIO DO CRONOGRAMA'!$E$5:$E$21</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="17"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
@@ -797,7 +2743,7 @@
                 <c:pt idx="5">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="8">
@@ -806,7 +2752,7 @@
                 <c:pt idx="9">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="12">
@@ -815,13 +2761,10 @@
                 <c:pt idx="13">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="15">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="17">
                   <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
@@ -1611,13 +3554,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1691640</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>3444240</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>28</xdr:row>
       <xdr:rowOff>160020</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2128,7 +4071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{541ADF72-36BD-4FF1-A5AB-A3492F022731}">
-  <dimension ref="B2:I23"/>
+  <dimension ref="B2:I22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
@@ -2137,41 +4080,41 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>23</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
@@ -2182,13 +4125,13 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0.5</v>
+        <v>13</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="6">
+        <v>1</v>
       </c>
       <c r="E6" s="3">
         <v>1</v>
@@ -2198,8 +4141,8 @@
       <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>25</v>
+      <c r="C7" s="22" t="s">
+        <v>23</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -2210,13 +4153,13 @@
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>23</v>
       </c>
       <c r="D8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="3">
         <v>1</v>
@@ -2224,10 +4167,10 @@
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>25</v>
+        <v>14</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>23</v>
       </c>
       <c r="D9" s="3">
         <v>1</v>
@@ -2238,46 +4181,46 @@
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>23</v>
       </c>
       <c r="D10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1</v>
-      </c>
+      <c r="B11" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B12" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>12</v>
       </c>
       <c r="D13" s="3">
         <v>0</v>
@@ -2288,47 +4231,47 @@
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="3">
+        <v>18</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="5">
         <v>0</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="6">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6">
-        <v>1</v>
-      </c>
+      <c r="B15" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="18"/>
+      <c r="I15" s="7"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B16" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="22"/>
-      <c r="I16" s="11"/>
+      <c r="B16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>12</v>
       </c>
       <c r="D17" s="3">
         <v>0</v>
@@ -2341,8 +4284,8 @@
       <c r="B18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>14</v>
+      <c r="C18" s="20" t="s">
+        <v>12</v>
       </c>
       <c r="D18" s="3">
         <v>0</v>
@@ -2352,92 +4295,57 @@
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="3">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3">
-        <v>1</v>
-      </c>
+      <c r="B19" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="18"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="22"/>
+      <c r="B20" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="9">
+        <v>0</v>
+      </c>
+      <c r="E20" s="9">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B21" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="13">
+      <c r="B21" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="3">
         <v>0</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B22" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D22" s="3">
-        <v>0</v>
-      </c>
-      <c r="E22" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B19:E19"/>
   </mergeCells>
-  <conditionalFormatting sqref="C6">
-    <cfRule type="containsText" dxfId="14" priority="15" operator="containsText" text="CONCLUIDA">
-      <formula>NOT(ISERROR(SEARCH("CONCLUIDA",C6)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="20" operator="containsText" text="PROGRESSO">
-      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C6)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="CONCLUIDA">
-      <formula>NOT(ISERROR(SEARCH("CONCLUIDA",C9)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="19" operator="containsText" text="PROGRESSO">
-      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C9)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C9 C17">
-    <cfRule type="containsText" dxfId="10" priority="18" operator="containsText" text="PROGRESSO">
-      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C6)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D6">
-    <cfRule type="dataBar" priority="17">
+  <conditionalFormatting sqref="D6 D8">
+    <cfRule type="dataBar" priority="26">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -2450,42 +4358,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D8:D9">
+  <conditionalFormatting sqref="D5:D10">
     <cfRule type="dataBar" priority="16">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="4" tint="0.59999389629810485"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B65D1A94-2492-4587-8A23-4A8E9AA1BA7B}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C5">
-    <cfRule type="containsText" dxfId="9" priority="14" operator="containsText" text="PROGRESSO">
-      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C10:C11">
-    <cfRule type="containsText" dxfId="8" priority="13" operator="containsText" text="PROGRESSO">
-      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C10)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C13:C15">
-    <cfRule type="containsText" dxfId="7" priority="12" operator="containsText" text="PROGRESSO">
-      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C13)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C8">
-    <cfRule type="containsText" dxfId="6" priority="9" operator="containsText" text="CONCLUIDA">
-      <formula>NOT(ISERROR(SEARCH("CONCLUIDA",C8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D5:D11">
-    <cfRule type="dataBar" priority="7">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -2497,7 +4371,7 @@
         </ext>
       </extLst>
     </cfRule>
-    <cfRule type="dataBar" priority="8">
+    <cfRule type="dataBar" priority="17">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -2510,34 +4384,25 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D15:E15">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
+  <conditionalFormatting sqref="D14:E14">
+    <cfRule type="cellIs" dxfId="4" priority="15" operator="equal">
       <formula>"PROGRESSO"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C13">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+  <conditionalFormatting sqref="C22">
+    <cfRule type="cellIs" dxfId="3" priority="10" operator="equal">
       <formula>"A FAZER"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C14:C15">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <formula>"A FAZER"</formula>
+  <conditionalFormatting sqref="J12 C12:C14 C16:C18 C20:C21 C5:C10">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="A FAZER">
+      <formula>NOT(ISERROR(SEARCH("A FAZER",C5)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C17:C19">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"A FAZER"</formula>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="PROGRESSO">
+      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C5)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="PROGRESSO">
-      <formula>NOT(ISERROR(SEARCH("PROGRESSO",C21)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C21:C23">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"A FAZER"</formula>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="CONCLUIDO">
+      <formula>NOT(ISERROR(SEARCH("CONCLUIDO",C5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2559,22 +4424,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D6</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B65D1A94-2492-4587-8A23-4A8E9AA1BA7B}">
-            <x14:dataBar minLength="0" maxLength="100">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D8:D9</xm:sqref>
+          <xm:sqref>D6 D8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{A20B9124-15F8-4C0E-845D-578B9C7AEA85}">
@@ -2601,7 +4451,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D5:D11</xm:sqref>
+          <xm:sqref>D5:D10</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>